<commit_message>
chore: checkpoint current ERP changes
</commit_message>
<xml_diff>
--- a/public/downloads/normal_1.xlsx
+++ b/public/downloads/normal_1.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="128">
   <si>
     <t xml:space="preserve">       东莞市方恩电子材料科技有限公司</t>
   </si>
@@ -123,6 +123,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="14"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>检</t>
     </r>
     <r>
@@ -185,16 +192,6 @@
       </rPr>
       <t>告</t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="14"/>
-        <rFont val="Times New Roman"/>
-        <charset val="134"/>
-      </rPr>
-      <t>11111</t>
-    </r>
   </si>
   <si>
     <r>
@@ -447,6 +444,21 @@
   </si>
   <si>
     <t>${width_standard}</t>
+  </si>
+  <si>
+    <t>${width_actual1}</t>
+  </si>
+  <si>
+    <t>${width_actual2}</t>
+  </si>
+  <si>
+    <t>${width_actual3}</t>
+  </si>
+  <si>
+    <t>${width_actual4}</t>
+  </si>
+  <si>
+    <t>${width_actual5}</t>
   </si>
   <si>
     <t>${width_result}</t>
@@ -1265,12 +1277,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="华文楷体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="9"/>
-      <name val="华文楷体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="华文楷体"/>
       <charset val="134"/>
     </font>
@@ -3226,16 +3238,26 @@
       <c r="D18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
+      <c r="E18" s="54" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="54" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="54" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="I18" s="54" t="s">
+        <v>44</v>
+      </c>
       <c r="J18" s="52" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K18" s="52" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L18" s="32"/>
     </row>
@@ -3244,32 +3266,32 @@
         <v>4</v>
       </c>
       <c r="B19" s="55" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="32" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E19" s="56" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F19" s="56" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G19" s="56" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H19" s="56" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="I19" s="56" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J19" s="52" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="K19" s="52" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="L19" s="32"/>
     </row>
@@ -3278,32 +3300,32 @@
         <v>5</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C20" s="49"/>
       <c r="D20" s="32" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E20" s="56" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G20" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="I20" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="J20" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="K20" s="52" t="s">
         <v>55</v>
-      </c>
-      <c r="H20" s="56" t="s">
-        <v>56</v>
-      </c>
-      <c r="I20" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="J20" s="52" t="s">
-        <v>58</v>
-      </c>
-      <c r="K20" s="52" t="s">
-        <v>50</v>
       </c>
       <c r="L20" s="32"/>
     </row>
@@ -3312,32 +3334,32 @@
         <v>6</v>
       </c>
       <c r="B21" s="48" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C21" s="49"/>
       <c r="D21" s="32" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E21" s="57" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F21" s="57" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G21" s="57" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H21" s="57" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I21" s="57" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J21" s="52" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K21" s="25" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L21" s="26"/>
     </row>
@@ -3346,24 +3368,24 @@
         <v>7</v>
       </c>
       <c r="B22" s="48" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C22" s="49"/>
       <c r="D22" s="52" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E22" s="58" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F22" s="59"/>
       <c r="G22" s="59"/>
       <c r="H22" s="59"/>
       <c r="I22" s="60"/>
       <c r="J22" s="52" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="K22" s="52" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L22" s="32"/>
     </row>
@@ -3372,32 +3394,32 @@
         <v>8</v>
       </c>
       <c r="B23" s="48" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C23" s="49"/>
       <c r="D23" s="61" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E23" s="62" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F23" s="62" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G23" s="62" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H23" s="62" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I23" s="54" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J23" s="52" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K23" s="25" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="L23" s="51"/>
     </row>
@@ -3406,24 +3428,24 @@
         <v>9</v>
       </c>
       <c r="B24" s="48" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C24" s="49"/>
       <c r="D24" s="52" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E24" s="63" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F24" s="64"/>
       <c r="G24" s="64"/>
       <c r="H24" s="64"/>
       <c r="I24" s="65"/>
       <c r="J24" s="52" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="K24" s="25" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L24" s="51"/>
     </row>
@@ -3432,24 +3454,24 @@
         <v>10</v>
       </c>
       <c r="B25" s="48" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C25" s="49"/>
       <c r="D25" s="52" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E25" s="63" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F25" s="64"/>
       <c r="G25" s="64"/>
       <c r="H25" s="64"/>
       <c r="I25" s="65"/>
       <c r="J25" s="52" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="K25" s="25" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="L25" s="51"/>
     </row>
@@ -3458,24 +3480,24 @@
         <v>11</v>
       </c>
       <c r="B26" s="48" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C26" s="49"/>
       <c r="D26" s="27" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E26" s="63" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F26" s="64"/>
       <c r="G26" s="64"/>
       <c r="H26" s="64"/>
       <c r="I26" s="65"/>
       <c r="J26" s="52" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="K26" s="66" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="L26" s="67"/>
     </row>
@@ -3484,24 +3506,24 @@
         <v>12</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="68" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E27" s="63" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="F27" s="64"/>
       <c r="G27" s="64"/>
       <c r="H27" s="64"/>
       <c r="I27" s="65"/>
       <c r="J27" s="52" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="L27" s="51"/>
     </row>
@@ -3510,24 +3532,24 @@
         <v>11</v>
       </c>
       <c r="B28" s="48" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C28" s="49"/>
       <c r="D28" s="69" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E28" s="69"/>
       <c r="F28" s="69"/>
       <c r="G28" s="69"/>
       <c r="H28" s="69"/>
       <c r="I28" s="69" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J28" s="52" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="K28" s="70" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="L28" s="71"/>
     </row>
@@ -3536,30 +3558,30 @@
         <v>12</v>
       </c>
       <c r="B29" s="48" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C29" s="49"/>
       <c r="D29" s="69" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E29" s="69"/>
       <c r="F29" s="69"/>
       <c r="G29" s="69"/>
       <c r="H29" s="69"/>
       <c r="I29" s="69" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="J29" s="52" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="K29" s="70" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="L29" s="71"/>
     </row>
     <row r="30" s="6" customFormat="1" ht="28" customHeight="1" spans="1:14">
       <c r="A30" s="72" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B30" s="73"/>
       <c r="C30" s="73"/>
@@ -3577,7 +3599,7 @@
     </row>
     <row r="31" s="6" customFormat="1" ht="28" customHeight="1" spans="1:14">
       <c r="A31" s="72" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B31" s="72"/>
       <c r="C31" s="72"/>
@@ -3595,7 +3617,7 @@
     </row>
     <row r="32" s="6" customFormat="1" ht="28" customHeight="1" spans="1:14">
       <c r="A32" s="72" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B32" s="73"/>
       <c r="C32" s="73"/>
@@ -3613,7 +3635,7 @@
     </row>
     <row r="33" s="6" customFormat="1" ht="28" customHeight="1" spans="1:20">
       <c r="A33" s="72" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B33" s="73"/>
       <c r="C33" s="73"/>
@@ -3631,7 +3653,7 @@
     </row>
     <row r="34" s="6" customFormat="1" ht="28" customHeight="1" spans="1:20">
       <c r="A34" s="76" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B34" s="76"/>
       <c r="C34" s="76"/>
@@ -3655,7 +3677,7 @@
     </row>
     <row r="35" s="6" customFormat="1" ht="28" customHeight="1" spans="1:20">
       <c r="A35" s="72" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B35" s="73"/>
       <c r="C35" s="73"/>
@@ -3689,27 +3711,27 @@
     </row>
     <row r="37" s="7" customFormat="1" ht="24" customHeight="1" spans="1:20">
       <c r="A37" s="78" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B37" s="79" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C37" s="78"/>
       <c r="D37" s="78"/>
       <c r="E37" s="78"/>
       <c r="F37" s="80" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G37" s="79" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H37" s="79"/>
       <c r="I37" s="80"/>
       <c r="J37" s="81" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K37" s="82" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L37" s="83"/>
     </row>

</xml_diff>